<commit_message>
Update RC history: add 2026 ПРОКАТ АНО МШК entry from history.xlsx
</commit_message>
<xml_diff>
--- a/pages/rc-app/history.xlsx
+++ b/pages/rc-app/history.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\_STUDY\RC_Structure\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\UU\UCampus\RC_Review\pages\rc-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AF020D-CE05-4802-B7A2-64489C224163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5B98EF-07F4-445B-A2D5-BDB7B455A333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="23500" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
+    <workbookView xWindow="38290" yWindow="-2750" windowWidth="38620" windowHeight="21100" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="24">
   <si>
     <t>РЦ</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>СТЕКЛОДУВНАЯ</t>
+  </si>
+  <si>
+    <t>ПРОКАТ АНО МШК</t>
   </si>
 </sst>
 </file>
@@ -464,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835D9306-4152-4C80-BC0E-FC58626EA9EA}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.54296875" customWidth="1"/>
@@ -671,24 +674,24 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>18</v>
@@ -698,10 +701,18 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="2">
+        <v>2030</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
@@ -841,6 +852,12 @@
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
     </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>